<commit_message>
Apply width clearance notes to Vertom screening
</commit_message>
<xml_diff>
--- a/vertom_convois_epr2.xlsx
+++ b/vertom_convois_epr2.xlsx
@@ -93,7 +93,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -120,12 +120,18 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -176,6 +182,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1661,7 +1670,7 @@
       </c>
       <c r="J20" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 1 hatch; fuel missing.</t>
+          <t>CANDIDATE: hold width 10.10 m; CE has 0.55 m each side; no tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -1713,7 +1722,7 @@
       </c>
       <c r="J21" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 1 hatch; fuel missing.</t>
+          <t>CANDIDATE: hold width 10.10 m; CE has 0.55 m each side; no tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
@@ -1765,7 +1774,7 @@
       </c>
       <c r="J22" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 1 hatch; fuel missing.</t>
+          <t>CANDIDATE: hold width 10.10 m; CE has 0.55 m each side; no tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -1973,7 +1982,7 @@
       </c>
       <c r="J26" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: partly tween deck; tanktop 17 t/m²; fuel missing.</t>
+          <t>CANDIDATE: hold width 13.20 m; width clearance passes; partly tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
@@ -2025,7 +2034,7 @@
       </c>
       <c r="J27" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: partly tween deck; tanktop 17 t/m²; fuel missing.</t>
+          <t>CANDIDATE: hold width 13.20 m; width clearance passes; partly tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
@@ -2077,7 +2086,7 @@
       </c>
       <c r="J28" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: partly tween deck; tanktop 17 t/m²; fuel missing.</t>
+          <t>CANDIDATE: hold width 13.20 m; width clearance passes; partly tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
@@ -3065,7 +3074,7 @@
       </c>
       <c r="J47" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 1 hatch; fuel missing.</t>
+          <t>CANDIDATE: hold width 12.60 m; width clearance passes; no tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="K47" s="5" t="inlineStr">
@@ -3117,7 +3126,7 @@
       </c>
       <c r="J48" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 1 hatch; fuel missing.</t>
+          <t>CANDIDATE: hold width 12.60 m; width clearance passes; no tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="K48" s="5" t="inlineStr">
@@ -3169,7 +3178,7 @@
       </c>
       <c r="J49" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 1 hatch; fuel missing.</t>
+          <t>CANDIDATE: hold width 12.60 m; width clearance passes; no tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="K49" s="5" t="inlineStr">
@@ -5561,7 +5570,7 @@
       </c>
       <c r="J95" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 6.3 t/day published; group fuel incomplete.</t>
+          <t>CANDIDATE: hold width 11.20 m; width clearance passes; no tween deck; 6.3 t/day published.</t>
         </is>
       </c>
       <c r="K95" s="5" t="inlineStr">
@@ -5613,7 +5622,7 @@
       </c>
       <c r="J96" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 6.3 t/day published; group fuel incomplete.</t>
+          <t>CANDIDATE: hold width 11.20 m; width clearance passes; no tween deck; 6.3 t/day published.</t>
         </is>
       </c>
       <c r="K96" s="5" t="inlineStr">
@@ -5665,7 +5674,7 @@
       </c>
       <c r="J97" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 6.3 t/day published; group fuel incomplete.</t>
+          <t>CANDIDATE: hold width 11.20 m; width clearance passes; no tween deck; 6.3 t/day published.</t>
         </is>
       </c>
       <c r="K97" s="5" t="inlineStr">
@@ -9149,7 +9158,7 @@
       </c>
       <c r="J164" s="12" t="inlineStr">
         <is>
-          <t>HOLD: full tween deck; open top 6.5 m &lt; GV 6.6 m; draft 8.03 m.</t>
+          <t>HOLD: hold width 15.20 m passes width; full tween deck; open top 6.5 m &lt; GV 6.6 m; draft 8.03 m.</t>
         </is>
       </c>
       <c r="K164" s="5" t="inlineStr">
@@ -9201,7 +9210,7 @@
       </c>
       <c r="J165" s="12" t="inlineStr">
         <is>
-          <t>HOLD: full tween deck; open top 6.5 m &lt; GV 6.6 m; draft 8.03 m.</t>
+          <t>HOLD: hold width 15.20 m passes width; full tween deck; open top 6.5 m &lt; GV 6.6 m; draft 8.03 m.</t>
         </is>
       </c>
       <c r="K165" s="5" t="inlineStr">
@@ -9253,7 +9262,7 @@
       </c>
       <c r="J166" s="12" t="inlineStr">
         <is>
-          <t>HOLD: full tween deck; open top 6.5 m &lt; GV 6.6 m; draft 8.03 m.</t>
+          <t>HOLD: hold width 15.20 m passes width; full tween deck; open top 6.5 m &lt; GV 6.6 m; draft 8.03 m.</t>
         </is>
       </c>
       <c r="K166" s="5" t="inlineStr">
@@ -9929,7 +9938,7 @@
       </c>
       <c r="J179" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 2 hatches; fuel missing.</t>
+          <t>CANDIDATE: hold width 12.70 m; width clearance passes; no tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="K179" s="5" t="inlineStr">
@@ -9981,7 +9990,7 @@
       </c>
       <c r="J180" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 2 hatches; fuel missing.</t>
+          <t>CANDIDATE: hold width 12.70 m; width clearance passes; no tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="K180" s="5" t="inlineStr">
@@ -10033,7 +10042,7 @@
       </c>
       <c r="J181" s="12" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 2 hatches; fuel missing.</t>
+          <t>CANDIDATE: hold width 12.70 m; width clearance passes; no tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="K181" s="5" t="inlineStr">
@@ -12428,7 +12437,7 @@
       </c>
       <c r="L8" s="14" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 1 hatch; fuel missing.</t>
+          <t>CANDIDATE: hold width 10.10 m; CE has 0.55 m each side; no tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="M8" s="15" t="inlineStr">
@@ -12530,7 +12539,7 @@
       </c>
       <c r="L10" s="14" t="inlineStr">
         <is>
-          <t>CANDIDATE: partly tween deck; tanktop 17 t/m²; fuel missing.</t>
+          <t>CANDIDATE: hold width 13.20 m; width clearance passes; partly tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="M10" s="15" t="inlineStr">
@@ -12887,7 +12896,7 @@
       </c>
       <c r="L17" s="14" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 1 hatch; fuel missing.</t>
+          <t>CANDIDATE: hold width 12.60 m; width clearance passes; no tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="M17" s="15" t="inlineStr">
@@ -13703,7 +13712,7 @@
       </c>
       <c r="L33" s="14" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 6.3 t/day published; group fuel incomplete.</t>
+          <t>CANDIDATE: hold width 11.20 m; width clearance passes; no tween deck; 6.3 t/day published.</t>
         </is>
       </c>
       <c r="M33" s="15" t="inlineStr">
@@ -14876,7 +14885,7 @@
       </c>
       <c r="L56" s="18" t="inlineStr">
         <is>
-          <t>HOLD: full tween deck; open top 6.5 m &lt; GV 6.6 m; draft 8.03 m.</t>
+          <t>HOLD: hold width 15.20 m passes width; full tween deck; open top 6.5 m &lt; GV 6.6 m; draft 8.03 m.</t>
         </is>
       </c>
       <c r="M56" s="19" t="inlineStr">
@@ -15131,7 +15140,7 @@
       </c>
       <c r="L61" s="14" t="inlineStr">
         <is>
-          <t>CANDIDATE: no tween deck; 2 hatches; fuel missing.</t>
+          <t>CANDIDATE: hold width 12.70 m; width clearance passes; no tween deck; fuel missing.</t>
         </is>
       </c>
       <c r="M61" s="15" t="inlineStr">
@@ -15790,7 +15799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -16125,7 +16134,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="24" t="inlineStr">
         <is>
           <t>1. Prefer a single-decker with no tween/intermediate deck.</t>
         </is>
@@ -16133,7 +16142,7 @@
       <c r="B32" s="23" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="24" t="inlineStr">
         <is>
           <t>2. If a tween deck exists, cargo must clear it or the deck must be removed/landed ashore.</t>
         </is>
@@ -16141,7 +16150,7 @@
       <c r="B33" s="23" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="24" t="inlineStr">
         <is>
           <t>3. Hatch opening and hold access must accept the cargo length and allow loading/unloading.</t>
         </is>
@@ -16149,7 +16158,7 @@
       <c r="B34" s="23" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" s="24" t="inlineStr">
         <is>
           <t>4. Cargo footprint must stay within the deck/tanktop rating; GV is about 3.61 t/m².</t>
         </is>
@@ -16157,7 +16166,7 @@
       <c r="B35" s="23" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="24" t="inlineStr">
         <is>
           <t>5. After deck, opening and load checks pass, choose the lowest published fuel consumption.</t>
         </is>
@@ -16165,7 +16174,7 @@
       <c r="B36" s="23" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="24" t="inlineStr">
         <is>
           <t>6. Draft above 7 m is a caution; maximum available depth is 12 m.</t>
         </is>
@@ -16173,12 +16182,24 @@
       <c r="B37" s="23" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" s="24" t="inlineStr">
         <is>
           <t>7. Missing deck/opening/fuel data means conditional, not final approval.</t>
         </is>
       </c>
       <c r="B38" s="23" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
+          <t>Vertom width-clearance check</t>
+        </is>
+      </c>
+      <c r="B40" s="21" t="inlineStr">
+        <is>
+          <t>For Vertom, require cargo width + 1.00 m (0.50 m each side) inside the published hold width; equal widths fail. Hatch clear widths are still unconfirmed.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>